<commit_message>
more new tools !
</commit_message>
<xml_diff>
--- a/other-files/student_tools.xlsx
+++ b/other-files/student_tools.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashle\Documents\GitHub\student-model-gallery\other-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A4FAEC-1033-4D98-B85D-A946A6727713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEDF51B9-AAA8-4F4E-9163-C5EA9E79A7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-48" yWindow="-48" windowWidth="23136" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -640,7 +640,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -950,6 +950,7 @@
       <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -1091,6 +1092,7 @@
       <c r="C17" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="D17" s="3"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -1169,6 +1171,7 @@
       <c r="C24" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="D24" s="3"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -1192,6 +1195,7 @@
       <c r="C26" s="1" t="s">
         <v>77</v>
       </c>
+      <c r="D26" s="3"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
@@ -1203,6 +1207,7 @@
       <c r="C27" s="1" t="s">
         <v>80</v>
       </c>
+      <c r="D27" s="3"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
@@ -1214,6 +1219,7 @@
       <c r="C28" s="1" t="s">
         <v>83</v>
       </c>
+      <c r="D28" s="3"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -1225,6 +1231,7 @@
       <c r="C29" s="1" t="s">
         <v>86</v>
       </c>
+      <c r="D29" s="3"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
@@ -1236,6 +1243,7 @@
       <c r="C30" s="1" t="s">
         <v>89</v>
       </c>
+      <c r="D30" s="3"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
@@ -1247,6 +1255,7 @@
       <c r="C31" s="1" t="s">
         <v>92</v>
       </c>
+      <c r="D31" s="3"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
@@ -1280,6 +1289,7 @@
       <c r="C34" s="1" t="s">
         <v>101</v>
       </c>
+      <c r="D34" s="3"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
@@ -1291,6 +1301,7 @@
       <c r="C35" s="1" t="s">
         <v>104</v>
       </c>
+      <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -1324,6 +1335,7 @@
       <c r="C38" s="1" t="s">
         <v>113</v>
       </c>
+      <c r="D38" s="3"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
@@ -1346,6 +1358,7 @@
       <c r="C40" s="1" t="s">
         <v>119</v>
       </c>
+      <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -1424,6 +1437,7 @@
       <c r="C47" s="1" t="s">
         <v>140</v>
       </c>
+      <c r="D47" s="3"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
@@ -1435,6 +1449,7 @@
       <c r="C48" s="1" t="s">
         <v>143</v>
       </c>
+      <c r="D48" s="3"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">

</xml_diff>